<commit_message>
Adding the piechart after all validation
</commit_message>
<xml_diff>
--- a/UPGRADED_Book1.xlsx
+++ b/UPGRADED_Book1.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidRows" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InvalidRows" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CleanedData" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -125,6 +126,85 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Validation Results</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$A$2:$A$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$2:$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -941,4 +1021,63 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Valid rows</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Invalid rows</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Validation run at</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:21:31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding the history to trace data
</commit_message>
<xml_diff>
--- a/UPGRADED_Book1.xlsx
+++ b/UPGRADED_Book1.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InvalidRows" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CleanedData" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -180,7 +181,170 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Validation History</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'History'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'History'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'History'!$C$2:$B$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'History'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'History'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'History'!$D$2:$C$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Run Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Row Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1072,8 +1236,53 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-23 22:21:31</t>
-        </is>
+          <t>2026-08-24 22:10:15</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Run Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valid Rows</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Invalid Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-24 22:10:15</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>